<commit_message>
Updated Excel workbooks in data processed folder
</commit_message>
<xml_diff>
--- a/data/processed/05_UC_Mock_Technical_Exercise_Brief.xlsx
+++ b/data/processed/05_UC_Mock_Technical_Exercise_Brief.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faith\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faith\Documents\UC_Service_Centre_Analysis\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62AA6738-3F0C-4181-BC4E-BB66482200C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D88FDD27-85DC-488D-9CB8-1C438180A075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exercise Brief" sheetId="1" r:id="rId1"/>
@@ -424,7 +424,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -444,6 +444,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -469,7 +475,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -477,9 +483,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -490,6 +493,11 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -812,7 +820,7 @@
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="90" customWidth="1"/>
+    <col min="3" max="3" width="136.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" ht="20.65">
@@ -835,124 +843,124 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
     </row>
-    <row r="6" spans="1:8" s="11" customFormat="1" ht="15" customHeight="1">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:8" s="10" customFormat="1" ht="15" customHeight="1">
+      <c r="A6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1">
+    <row r="7" spans="1:8" ht="29.25" customHeight="1">
       <c r="A7" s="5">
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1">
+    <row r="8" spans="1:8" ht="29.25" customHeight="1">
       <c r="A8" s="5">
         <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="24" customHeight="1">
+    <row r="9" spans="1:8" ht="29.25" customHeight="1">
       <c r="A9" s="5">
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="24" customHeight="1">
+    <row r="10" spans="1:8" ht="29.25" customHeight="1">
       <c r="A10" s="5">
         <v>4</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1">
+    <row r="11" spans="1:8" ht="29.25" customHeight="1">
       <c r="A11" s="5">
         <v>5</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="24" customHeight="1">
+    <row r="12" spans="1:8" ht="29.25" customHeight="1">
       <c r="A12" s="5">
         <v>6</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1">
+    <row r="13" spans="1:8" ht="29.25" customHeight="1">
       <c r="A13" s="5">
         <v>7</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="11" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1">
+    <row r="14" spans="1:8" ht="29.25" customHeight="1">
       <c r="A14" s="5">
         <v>8</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="11" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15" customHeight="1">
+    <row r="15" spans="1:8" ht="29.25" customHeight="1">
       <c r="A15" s="5">
         <v>9</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1">
-      <c r="A16">
+    <row r="16" spans="1:8" ht="29.25" customHeight="1">
+      <c r="A16" s="5">
         <v>10</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="11" t="s">
         <v>38</v>
       </c>
     </row>
@@ -973,268 +981,268 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="18" customHeight="1">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="18" customHeight="1">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="18" customHeight="1">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="18" customHeight="1">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="18" customHeight="1">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="7" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="18" customHeight="1">
-      <c r="A15" s="8" t="s">
+    <row r="15" spans="1:4" s="13" customFormat="1" ht="18" customHeight="1">
+      <c r="A15" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="12" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="7" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="18" customHeight="1">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="7" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="18" customHeight="1">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="7" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="18" customHeight="1">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="7" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1257,101 +1265,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="18" customHeight="1">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" customHeight="1">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="18" customHeight="1">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="18" customHeight="1">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="18" customHeight="1">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="18" customHeight="1">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="18" customHeight="1">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="18" customHeight="1">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>117</v>
       </c>
     </row>

</xml_diff>